<commit_message>
fix: KPI cards filter policy table (not flags page), normalize flag names, add Suspense boundaries for all useSearchParams pages, move analytics above table (default open)
</commit_message>
<xml_diff>
--- a/Copy of CoverageCheckNow_Flag_Definitions.xlsx
+++ b/Copy of CoverageCheckNow_Flag_Definitions.xlsx
@@ -3,14 +3,15 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FBCE93C4-5C69-4345-B4B7-18B958FFD4F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10A7179F-DEEC-4F7E-A906-C71A423F20EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-2715" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Flag Definitions" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1659,7 +1660,7 @@
     <col min="17" max="17" width="26.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="1" customFormat="1" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" s="1" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1757,7 +1758,7 @@
       </c>
       <c r="P2" s="9"/>
     </row>
-    <row r="3" spans="1:17" s="2" customFormat="1" ht="36" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" s="2" customFormat="1" ht="72" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>

</xml_diff>